<commit_message>
Chicago: hoja única carta imprimible (2 columnas), orden alfabético, +Arrachera, línea de fecha
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mmrn7JLAhSVspHUWxCQFPE
</commit_message>
<xml_diff>
--- a/CHICAGO DEEP DISH PIZZA/Existencias_Diarias_Chicago.xlsx
+++ b/CHICAGO DEEP DISH PIZZA/Existencias_Diarias_Chicago.xlsx
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D141"/>
+  <dimension ref="A1:D142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -749,7 +749,7 @@
     <row r="16" ht="17" customHeight="1">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>Chile Serrano</t>
+          <t>Chile Guajillo</t>
         </is>
       </c>
       <c r="B16" s="11" t="n"/>
@@ -759,7 +759,7 @@
     <row r="17" ht="17" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>Chile Guajillo</t>
+          <t>Chile Jalapeño</t>
         </is>
       </c>
       <c r="B17" s="11" t="n"/>
@@ -769,7 +769,7 @@
     <row r="18" ht="17" customHeight="1">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>Chile Jalapeño</t>
+          <t>Chile Morita</t>
         </is>
       </c>
       <c r="B18" s="11" t="n"/>
@@ -779,7 +779,7 @@
     <row r="19" ht="17" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>Chile Morita</t>
+          <t>Chile Serrano</t>
         </is>
       </c>
       <c r="B19" s="11" t="n"/>
@@ -879,7 +879,7 @@
     <row r="29" ht="17" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>Pimiento</t>
+          <t>Orégano</t>
         </is>
       </c>
       <c r="B29" s="11" t="n"/>
@@ -889,7 +889,7 @@
     <row r="30" ht="17" customHeight="1">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>Orégano</t>
+          <t>Pimiento</t>
         </is>
       </c>
       <c r="B30" s="11" t="n"/>
@@ -951,7 +951,7 @@
     <row r="37" ht="17" customHeight="1">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>BBQ</t>
+          <t>Arrachera</t>
         </is>
       </c>
       <c r="B37" s="11" t="n"/>
@@ -961,7 +961,7 @@
     <row r="38" ht="17" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>Boneless</t>
+          <t>BBQ</t>
         </is>
       </c>
       <c r="B38" s="11" t="n"/>
@@ -971,7 +971,7 @@
     <row r="39" ht="17" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>Búfalo</t>
+          <t>Boneless</t>
         </is>
       </c>
       <c r="B39" s="11" t="n"/>
@@ -981,7 +981,7 @@
     <row r="40" ht="17" customHeight="1">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>Calamares</t>
+          <t>Búfalo</t>
         </is>
       </c>
       <c r="B40" s="11" t="n"/>
@@ -991,7 +991,7 @@
     <row r="41" ht="17" customHeight="1">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>Camarón</t>
+          <t>Calamares</t>
         </is>
       </c>
       <c r="B41" s="11" t="n"/>
@@ -1001,7 +1001,7 @@
     <row r="42" ht="17" customHeight="1">
       <c r="A42" s="10" t="inlineStr">
         <is>
-          <t>Carne Molida</t>
+          <t>Camarón</t>
         </is>
       </c>
       <c r="B42" s="11" t="n"/>
@@ -1011,7 +1011,7 @@
     <row r="43" ht="17" customHeight="1">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>Chistorra</t>
+          <t>Carne Molida</t>
         </is>
       </c>
       <c r="B43" s="11" t="n"/>
@@ -1021,7 +1021,7 @@
     <row r="44" ht="17" customHeight="1">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Dedos de Queso</t>
+          <t>Chistorra</t>
         </is>
       </c>
       <c r="B44" s="11" t="n"/>
@@ -1031,7 +1031,7 @@
     <row r="45" ht="17" customHeight="1">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>Pan</t>
+          <t>Dedos de Queso</t>
         </is>
       </c>
       <c r="B45" s="11" t="n"/>
@@ -1051,7 +1051,7 @@
     <row r="47" ht="17" customHeight="1">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>Papas a la Francesa</t>
+          <t>Pan</t>
         </is>
       </c>
       <c r="B47" s="11" t="n"/>
@@ -1061,7 +1061,7 @@
     <row r="48" ht="17" customHeight="1">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>Pepperoni</t>
+          <t>Papas a la Francesa</t>
         </is>
       </c>
       <c r="B48" s="11" t="n"/>
@@ -1071,7 +1071,7 @@
     <row r="49" ht="17" customHeight="1">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>Ranch</t>
+          <t>Pepperoni</t>
         </is>
       </c>
       <c r="B49" s="11" t="n"/>
@@ -1081,7 +1081,7 @@
     <row r="50" ht="17" customHeight="1">
       <c r="A50" s="10" t="inlineStr">
         <is>
-          <t>Salami</t>
+          <t>Ranch</t>
         </is>
       </c>
       <c r="B50" s="11" t="n"/>
@@ -1091,7 +1091,7 @@
     <row r="51" ht="17" customHeight="1">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>Salchicha Italiana</t>
+          <t>Salami</t>
         </is>
       </c>
       <c r="B51" s="11" t="n"/>
@@ -1101,7 +1101,7 @@
     <row r="52" ht="17" customHeight="1">
       <c r="A52" s="10" t="inlineStr">
         <is>
-          <t>Tocino</t>
+          <t>Salchicha Italiana</t>
         </is>
       </c>
       <c r="B52" s="11" t="n"/>
@@ -1109,7 +1109,11 @@
       <c r="D52" s="12" t="n"/>
     </row>
     <row r="53" ht="17" customHeight="1">
-      <c r="A53" s="13" t="inlineStr"/>
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>Tocino</t>
+        </is>
+      </c>
       <c r="B53" s="11" t="n"/>
       <c r="C53" s="11" t="n"/>
       <c r="D53" s="14" t="n"/>
@@ -1120,872 +1124,878 @@
       <c r="C54" s="11" t="n"/>
       <c r="D54" s="12" t="n"/>
     </row>
-    <row r="55" ht="19" customHeight="1">
-      <c r="A55" s="8" t="inlineStr">
+    <row r="55" ht="17" customHeight="1">
+      <c r="A55" s="13" t="inlineStr"/>
+      <c r="B55" s="11" t="n"/>
+      <c r="C55" s="11" t="n"/>
+      <c r="D55" s="14" t="n"/>
+    </row>
+    <row r="56" ht="19" customHeight="1">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>ALMACÉN</t>
         </is>
       </c>
-      <c r="B55" s="9" t="n"/>
-      <c r="C55" s="9" t="n"/>
-      <c r="D55" s="9" t="n"/>
-    </row>
-    <row r="56" ht="17" customHeight="1">
-      <c r="A56" s="10" t="inlineStr">
+      <c r="B56" s="9" t="n"/>
+      <c r="C56" s="9" t="n"/>
+      <c r="D56" s="9" t="n"/>
+    </row>
+    <row r="57" ht="17" customHeight="1">
+      <c r="A57" s="10" t="inlineStr">
         <is>
           <t>Aceite</t>
-        </is>
-      </c>
-      <c r="B56" s="11" t="n"/>
-      <c r="C56" s="11" t="n"/>
-      <c r="D56" s="12" t="n"/>
-    </row>
-    <row r="57" ht="17" customHeight="1">
-      <c r="A57" s="13" t="inlineStr">
-        <is>
-          <t>Aceite freidora</t>
         </is>
       </c>
       <c r="B57" s="11" t="n"/>
       <c r="C57" s="11" t="n"/>
-      <c r="D57" s="14" t="n"/>
+      <c r="D57" s="12" t="n"/>
     </row>
     <row r="58" ht="17" customHeight="1">
-      <c r="A58" s="10" t="inlineStr">
+      <c r="A58" s="13" t="inlineStr">
         <is>
           <t>Aceite de Oliva</t>
         </is>
       </c>
       <c r="B58" s="11" t="n"/>
       <c r="C58" s="11" t="n"/>
-      <c r="D58" s="12" t="n"/>
+      <c r="D58" s="14" t="n"/>
     </row>
     <row r="59" ht="17" customHeight="1">
-      <c r="A59" s="13" t="inlineStr">
-        <is>
-          <t>Aceituna negra</t>
+      <c r="A59" s="10" t="inlineStr">
+        <is>
+          <t>Aceite freidora</t>
         </is>
       </c>
       <c r="B59" s="11" t="n"/>
       <c r="C59" s="11" t="n"/>
-      <c r="D59" s="14" t="n"/>
+      <c r="D59" s="12" t="n"/>
     </row>
     <row r="60" ht="17" customHeight="1">
-      <c r="A60" s="10" t="inlineStr">
-        <is>
-          <t>Ajo en Polvo</t>
+      <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>Aceituna negra</t>
         </is>
       </c>
       <c r="B60" s="11" t="n"/>
       <c r="C60" s="11" t="n"/>
-      <c r="D60" s="12" t="n"/>
+      <c r="D60" s="14" t="n"/>
     </row>
     <row r="61" ht="17" customHeight="1">
-      <c r="A61" s="13" t="inlineStr">
-        <is>
-          <t>Albahaca Deshidratada</t>
+      <c r="A61" s="10" t="inlineStr">
+        <is>
+          <t>Ajo en Polvo</t>
         </is>
       </c>
       <c r="B61" s="11" t="n"/>
       <c r="C61" s="11" t="n"/>
-      <c r="D61" s="14" t="n"/>
+      <c r="D61" s="12" t="n"/>
     </row>
     <row r="62" ht="17" customHeight="1">
-      <c r="A62" s="10" t="inlineStr">
-        <is>
-          <t>Alcachofa</t>
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>Albahaca Deshidratada</t>
         </is>
       </c>
       <c r="B62" s="11" t="n"/>
       <c r="C62" s="11" t="n"/>
-      <c r="D62" s="12" t="n"/>
+      <c r="D62" s="14" t="n"/>
     </row>
     <row r="63" ht="17" customHeight="1">
-      <c r="A63" s="13" t="inlineStr">
-        <is>
-          <t>Aluminio</t>
+      <c r="A63" s="10" t="inlineStr">
+        <is>
+          <t>Alcachofa</t>
         </is>
       </c>
       <c r="B63" s="11" t="n"/>
       <c r="C63" s="11" t="n"/>
-      <c r="D63" s="14" t="n"/>
+      <c r="D63" s="12" t="n"/>
     </row>
     <row r="64" ht="17" customHeight="1">
-      <c r="A64" s="10" t="inlineStr">
-        <is>
-          <t>Anís Estrella</t>
+      <c r="A64" s="13" t="inlineStr">
+        <is>
+          <t>Aluminio</t>
         </is>
       </c>
       <c r="B64" s="11" t="n"/>
       <c r="C64" s="11" t="n"/>
-      <c r="D64" s="12" t="n"/>
+      <c r="D64" s="14" t="n"/>
     </row>
     <row r="65" ht="17" customHeight="1">
-      <c r="A65" s="13" t="inlineStr">
-        <is>
-          <t>Arándanos</t>
+      <c r="A65" s="10" t="inlineStr">
+        <is>
+          <t>Anís Estrella</t>
         </is>
       </c>
       <c r="B65" s="11" t="n"/>
       <c r="C65" s="11" t="n"/>
-      <c r="D65" s="14" t="n"/>
+      <c r="D65" s="12" t="n"/>
     </row>
     <row r="66" ht="17" customHeight="1">
-      <c r="A66" s="10" t="inlineStr">
-        <is>
-          <t>Azúcar</t>
+      <c r="A66" s="13" t="inlineStr">
+        <is>
+          <t>Arándanos</t>
         </is>
       </c>
       <c r="B66" s="11" t="n"/>
       <c r="C66" s="11" t="n"/>
-      <c r="D66" s="12" t="n"/>
+      <c r="D66" s="14" t="n"/>
     </row>
     <row r="67" ht="17" customHeight="1">
-      <c r="A67" s="13" t="inlineStr">
-        <is>
-          <t>Bactericida</t>
+      <c r="A67" s="10" t="inlineStr">
+        <is>
+          <t>Azúcar</t>
         </is>
       </c>
       <c r="B67" s="11" t="n"/>
       <c r="C67" s="11" t="n"/>
-      <c r="D67" s="14" t="n"/>
+      <c r="D67" s="12" t="n"/>
     </row>
     <row r="68" ht="17" customHeight="1">
-      <c r="A68" s="10" t="inlineStr">
-        <is>
-          <t>Cacahuate</t>
+      <c r="A68" s="13" t="inlineStr">
+        <is>
+          <t>Bactericida</t>
         </is>
       </c>
       <c r="B68" s="11" t="n"/>
       <c r="C68" s="11" t="n"/>
-      <c r="D68" s="12" t="n"/>
+      <c r="D68" s="14" t="n"/>
     </row>
     <row r="69" ht="17" customHeight="1">
-      <c r="A69" s="13" t="inlineStr">
-        <is>
-          <t>Cardamomo</t>
+      <c r="A69" s="10" t="inlineStr">
+        <is>
+          <t>Cacahuate</t>
         </is>
       </c>
       <c r="B69" s="11" t="n"/>
       <c r="C69" s="11" t="n"/>
-      <c r="D69" s="14" t="n"/>
+      <c r="D69" s="12" t="n"/>
     </row>
     <row r="70" ht="17" customHeight="1">
-      <c r="A70" s="10" t="inlineStr">
-        <is>
-          <t>Catsup</t>
+      <c r="A70" s="13" t="inlineStr">
+        <is>
+          <t>Cardamomo</t>
         </is>
       </c>
       <c r="B70" s="11" t="n"/>
       <c r="C70" s="11" t="n"/>
-      <c r="D70" s="12" t="n"/>
+      <c r="D70" s="14" t="n"/>
     </row>
     <row r="71" ht="17" customHeight="1">
-      <c r="A71" s="13" t="inlineStr">
-        <is>
-          <t>Cebolla en Polvo</t>
+      <c r="A71" s="10" t="inlineStr">
+        <is>
+          <t>Catsup</t>
         </is>
       </c>
       <c r="B71" s="11" t="n"/>
       <c r="C71" s="11" t="n"/>
-      <c r="D71" s="14" t="n"/>
+      <c r="D71" s="12" t="n"/>
     </row>
     <row r="72" ht="17" customHeight="1">
-      <c r="A72" s="10" t="inlineStr">
-        <is>
-          <t>Chipotle</t>
+      <c r="A72" s="13" t="inlineStr">
+        <is>
+          <t>Cebolla en Polvo</t>
         </is>
       </c>
       <c r="B72" s="11" t="n"/>
       <c r="C72" s="11" t="n"/>
-      <c r="D72" s="12" t="n"/>
+      <c r="D72" s="14" t="n"/>
     </row>
     <row r="73" ht="17" customHeight="1">
-      <c r="A73" s="13" t="inlineStr">
-        <is>
-          <t>Chocolate</t>
+      <c r="A73" s="10" t="inlineStr">
+        <is>
+          <t>Chipotle</t>
         </is>
       </c>
       <c r="B73" s="11" t="n"/>
       <c r="C73" s="11" t="n"/>
-      <c r="D73" s="14" t="n"/>
+      <c r="D73" s="12" t="n"/>
     </row>
     <row r="74" ht="17" customHeight="1">
-      <c r="A74" s="10" t="inlineStr">
-        <is>
-          <t>Clavo</t>
+      <c r="A74" s="13" t="inlineStr">
+        <is>
+          <t>Chocolate</t>
         </is>
       </c>
       <c r="B74" s="11" t="n"/>
       <c r="C74" s="11" t="n"/>
-      <c r="D74" s="12" t="n"/>
+      <c r="D74" s="14" t="n"/>
     </row>
     <row r="75" ht="17" customHeight="1">
-      <c r="A75" s="13" t="inlineStr">
-        <is>
-          <t>Condimento Italiano</t>
+      <c r="A75" s="10" t="inlineStr">
+        <is>
+          <t>Clavo</t>
         </is>
       </c>
       <c r="B75" s="11" t="n"/>
       <c r="C75" s="11" t="n"/>
-      <c r="D75" s="14" t="n"/>
+      <c r="D75" s="12" t="n"/>
     </row>
     <row r="76" ht="17" customHeight="1">
-      <c r="A76" s="10" t="inlineStr">
-        <is>
-          <t>Consomé</t>
+      <c r="A76" s="13" t="inlineStr">
+        <is>
+          <t>Condimento Italiano</t>
         </is>
       </c>
       <c r="B76" s="11" t="n"/>
       <c r="C76" s="11" t="n"/>
-      <c r="D76" s="12" t="n"/>
+      <c r="D76" s="14" t="n"/>
     </row>
     <row r="77" ht="17" customHeight="1">
-      <c r="A77" s="13" t="inlineStr">
-        <is>
-          <t>Crema para Batir</t>
+      <c r="A77" s="10" t="inlineStr">
+        <is>
+          <t>Consomé</t>
         </is>
       </c>
       <c r="B77" s="11" t="n"/>
       <c r="C77" s="11" t="n"/>
-      <c r="D77" s="14" t="n"/>
+      <c r="D77" s="12" t="n"/>
     </row>
     <row r="78" ht="17" customHeight="1">
-      <c r="A78" s="10" t="inlineStr">
-        <is>
-          <t>Espagueti</t>
+      <c r="A78" s="13" t="inlineStr">
+        <is>
+          <t>Crema para Batir</t>
         </is>
       </c>
       <c r="B78" s="11" t="n"/>
       <c r="C78" s="11" t="n"/>
-      <c r="D78" s="12" t="n"/>
+      <c r="D78" s="14" t="n"/>
     </row>
     <row r="79" ht="17" customHeight="1">
-      <c r="A79" s="13" t="inlineStr">
-        <is>
-          <t>Frutos rojos</t>
+      <c r="A79" s="10" t="inlineStr">
+        <is>
+          <t>Espagueti</t>
         </is>
       </c>
       <c r="B79" s="11" t="n"/>
       <c r="C79" s="11" t="n"/>
-      <c r="D79" s="14" t="n"/>
+      <c r="D79" s="12" t="n"/>
     </row>
     <row r="80" ht="17" customHeight="1">
-      <c r="A80" s="10" t="inlineStr">
-        <is>
-          <t>Grenetina</t>
+      <c r="A80" s="13" t="inlineStr">
+        <is>
+          <t>Frutos rojos</t>
         </is>
       </c>
       <c r="B80" s="11" t="n"/>
       <c r="C80" s="11" t="n"/>
-      <c r="D80" s="12" t="n"/>
+      <c r="D80" s="14" t="n"/>
     </row>
     <row r="81" ht="17" customHeight="1">
-      <c r="A81" s="13" t="inlineStr">
-        <is>
-          <t>Harina</t>
+      <c r="A81" s="10" t="inlineStr">
+        <is>
+          <t>Grenetina</t>
         </is>
       </c>
       <c r="B81" s="11" t="n"/>
       <c r="C81" s="11" t="n"/>
-      <c r="D81" s="14" t="n"/>
+      <c r="D81" s="12" t="n"/>
     </row>
     <row r="82" ht="17" customHeight="1">
-      <c r="A82" s="10" t="inlineStr">
-        <is>
-          <t>Harina de arroz</t>
+      <c r="A82" s="13" t="inlineStr">
+        <is>
+          <t>Harina</t>
         </is>
       </c>
       <c r="B82" s="11" t="n"/>
       <c r="C82" s="11" t="n"/>
-      <c r="D82" s="12" t="n"/>
+      <c r="D82" s="14" t="n"/>
     </row>
     <row r="83" ht="17" customHeight="1">
-      <c r="A83" s="13" t="inlineStr">
-        <is>
-          <t>Hojaldra</t>
+      <c r="A83" s="10" t="inlineStr">
+        <is>
+          <t>Harina de arroz</t>
         </is>
       </c>
       <c r="B83" s="11" t="n"/>
       <c r="C83" s="11" t="n"/>
-      <c r="D83" s="14" t="n"/>
+      <c r="D83" s="12" t="n"/>
     </row>
     <row r="84" ht="17" customHeight="1">
-      <c r="A84" s="10" t="inlineStr">
-        <is>
-          <t>Jamón Serrano</t>
+      <c r="A84" s="13" t="inlineStr">
+        <is>
+          <t>Hojaldra</t>
         </is>
       </c>
       <c r="B84" s="11" t="n"/>
       <c r="C84" s="11" t="n"/>
-      <c r="D84" s="12" t="n"/>
+      <c r="D84" s="14" t="n"/>
     </row>
     <row r="85" ht="17" customHeight="1">
-      <c r="A85" s="13" t="inlineStr">
-        <is>
-          <t>Leche evaporada</t>
+      <c r="A85" s="10" t="inlineStr">
+        <is>
+          <t>Jamón Serrano</t>
         </is>
       </c>
       <c r="B85" s="11" t="n"/>
       <c r="C85" s="11" t="n"/>
-      <c r="D85" s="14" t="n"/>
+      <c r="D85" s="12" t="n"/>
     </row>
     <row r="86" ht="17" customHeight="1">
-      <c r="A86" s="10" t="inlineStr">
+      <c r="A86" s="13" t="inlineStr">
         <is>
           <t>Leche Entera</t>
         </is>
       </c>
       <c r="B86" s="11" t="n"/>
       <c r="C86" s="11" t="n"/>
-      <c r="D86" s="12" t="n"/>
+      <c r="D86" s="14" t="n"/>
     </row>
     <row r="87" ht="17" customHeight="1">
-      <c r="A87" s="13" t="inlineStr">
-        <is>
-          <t>Lemon Pepper</t>
+      <c r="A87" s="10" t="inlineStr">
+        <is>
+          <t>Leche evaporada</t>
         </is>
       </c>
       <c r="B87" s="11" t="n"/>
       <c r="C87" s="11" t="n"/>
-      <c r="D87" s="14" t="n"/>
+      <c r="D87" s="12" t="n"/>
     </row>
     <row r="88" ht="17" customHeight="1">
-      <c r="A88" s="10" t="inlineStr">
-        <is>
-          <t>Levadura</t>
+      <c r="A88" s="13" t="inlineStr">
+        <is>
+          <t>Lemon Pepper</t>
         </is>
       </c>
       <c r="B88" s="11" t="n"/>
       <c r="C88" s="11" t="n"/>
-      <c r="D88" s="12" t="n"/>
+      <c r="D88" s="14" t="n"/>
     </row>
     <row r="89" ht="17" customHeight="1">
-      <c r="A89" s="13" t="inlineStr">
-        <is>
-          <t>Maizena</t>
+      <c r="A89" s="10" t="inlineStr">
+        <is>
+          <t>Levadura</t>
         </is>
       </c>
       <c r="B89" s="11" t="n"/>
       <c r="C89" s="11" t="n"/>
-      <c r="D89" s="14" t="n"/>
+      <c r="D89" s="12" t="n"/>
     </row>
     <row r="90" ht="17" customHeight="1">
-      <c r="A90" s="10" t="inlineStr">
-        <is>
-          <t>Margarina</t>
+      <c r="A90" s="13" t="inlineStr">
+        <is>
+          <t>Maizena</t>
         </is>
       </c>
       <c r="B90" s="11" t="n"/>
       <c r="C90" s="11" t="n"/>
-      <c r="D90" s="12" t="n"/>
+      <c r="D90" s="14" t="n"/>
     </row>
     <row r="91" ht="17" customHeight="1">
-      <c r="A91" s="13" t="inlineStr">
-        <is>
-          <t>Mayonesa</t>
+      <c r="A91" s="10" t="inlineStr">
+        <is>
+          <t>Margarina</t>
         </is>
       </c>
       <c r="B91" s="11" t="n"/>
       <c r="C91" s="11" t="n"/>
-      <c r="D91" s="14" t="n"/>
+      <c r="D91" s="12" t="n"/>
     </row>
     <row r="92" ht="17" customHeight="1">
-      <c r="A92" s="10" t="inlineStr">
-        <is>
-          <t>Media crema</t>
+      <c r="A92" s="13" t="inlineStr">
+        <is>
+          <t>Mayonesa</t>
         </is>
       </c>
       <c r="B92" s="11" t="n"/>
       <c r="C92" s="11" t="n"/>
-      <c r="D92" s="12" t="n"/>
+      <c r="D92" s="14" t="n"/>
     </row>
     <row r="93" ht="17" customHeight="1">
-      <c r="A93" s="13" t="inlineStr">
-        <is>
-          <t>Miel</t>
+      <c r="A93" s="10" t="inlineStr">
+        <is>
+          <t>Media crema</t>
         </is>
       </c>
       <c r="B93" s="11" t="n"/>
       <c r="C93" s="11" t="n"/>
-      <c r="D93" s="14" t="n"/>
+      <c r="D93" s="12" t="n"/>
     </row>
     <row r="94" ht="17" customHeight="1">
-      <c r="A94" s="10" t="inlineStr">
-        <is>
-          <t>Mostaza</t>
+      <c r="A94" s="13" t="inlineStr">
+        <is>
+          <t>Miel</t>
         </is>
       </c>
       <c r="B94" s="11" t="n"/>
       <c r="C94" s="11" t="n"/>
-      <c r="D94" s="12" t="n"/>
+      <c r="D94" s="14" t="n"/>
     </row>
     <row r="95" ht="17" customHeight="1">
-      <c r="A95" s="13" t="inlineStr">
-        <is>
-          <t>Nuez Caramelizada</t>
+      <c r="A95" s="10" t="inlineStr">
+        <is>
+          <t>Mostaza</t>
         </is>
       </c>
       <c r="B95" s="11" t="n"/>
       <c r="C95" s="11" t="n"/>
-      <c r="D95" s="14" t="n"/>
+      <c r="D95" s="12" t="n"/>
     </row>
     <row r="96" ht="17" customHeight="1">
-      <c r="A96" s="10" t="inlineStr">
-        <is>
-          <t>Ostiones</t>
+      <c r="A96" s="13" t="inlineStr">
+        <is>
+          <t>Nuez Caramelizada</t>
         </is>
       </c>
       <c r="B96" s="11" t="n"/>
       <c r="C96" s="11" t="n"/>
-      <c r="D96" s="12" t="n"/>
+      <c r="D96" s="14" t="n"/>
     </row>
     <row r="97" ht="17" customHeight="1">
-      <c r="A97" s="13" t="inlineStr">
-        <is>
-          <t>Paprika</t>
+      <c r="A97" s="10" t="inlineStr">
+        <is>
+          <t>Ostiones</t>
         </is>
       </c>
       <c r="B97" s="11" t="n"/>
       <c r="C97" s="11" t="n"/>
-      <c r="D97" s="14" t="n"/>
+      <c r="D97" s="12" t="n"/>
     </row>
     <row r="98" ht="17" customHeight="1">
-      <c r="A98" s="10" t="inlineStr">
-        <is>
-          <t>Pimienta trozada</t>
+      <c r="A98" s="13" t="inlineStr">
+        <is>
+          <t>Paprika</t>
         </is>
       </c>
       <c r="B98" s="11" t="n"/>
       <c r="C98" s="11" t="n"/>
-      <c r="D98" s="12" t="n"/>
+      <c r="D98" s="14" t="n"/>
     </row>
     <row r="99" ht="17" customHeight="1">
-      <c r="A99" s="13" t="inlineStr">
-        <is>
-          <t>Pimiento Morrón</t>
+      <c r="A99" s="10" t="inlineStr">
+        <is>
+          <t>Pimienta trozada</t>
         </is>
       </c>
       <c r="B99" s="11" t="n"/>
       <c r="C99" s="11" t="n"/>
-      <c r="D99" s="14" t="n"/>
+      <c r="D99" s="12" t="n"/>
     </row>
     <row r="100" ht="17" customHeight="1">
-      <c r="A100" s="10" t="inlineStr">
-        <is>
-          <t>Piña</t>
+      <c r="A100" s="13" t="inlineStr">
+        <is>
+          <t>Pimiento Morrón</t>
         </is>
       </c>
       <c r="B100" s="11" t="n"/>
       <c r="C100" s="11" t="n"/>
-      <c r="D100" s="12" t="n"/>
+      <c r="D100" s="14" t="n"/>
     </row>
     <row r="101" ht="17" customHeight="1">
-      <c r="A101" s="13" t="inlineStr">
-        <is>
-          <t>Queso Amarillo</t>
+      <c r="A101" s="10" t="inlineStr">
+        <is>
+          <t>Piña</t>
         </is>
       </c>
       <c r="B101" s="11" t="n"/>
       <c r="C101" s="11" t="n"/>
-      <c r="D101" s="14" t="n"/>
+      <c r="D101" s="12" t="n"/>
     </row>
     <row r="102" ht="17" customHeight="1">
-      <c r="A102" s="10" t="inlineStr">
-        <is>
-          <t>Queso Cabra</t>
+      <c r="A102" s="13" t="inlineStr">
+        <is>
+          <t>Queso Amarillo</t>
         </is>
       </c>
       <c r="B102" s="11" t="n"/>
       <c r="C102" s="11" t="n"/>
-      <c r="D102" s="12" t="n"/>
+      <c r="D102" s="14" t="n"/>
     </row>
     <row r="103" ht="17" customHeight="1">
-      <c r="A103" s="13" t="inlineStr">
-        <is>
-          <t>Queso Crema</t>
+      <c r="A103" s="10" t="inlineStr">
+        <is>
+          <t>Queso Cabra</t>
         </is>
       </c>
       <c r="B103" s="11" t="n"/>
       <c r="C103" s="11" t="n"/>
-      <c r="D103" s="14" t="n"/>
+      <c r="D103" s="12" t="n"/>
     </row>
     <row r="104" ht="17" customHeight="1">
-      <c r="A104" s="10" t="inlineStr">
-        <is>
-          <t>Queso Mozzarella</t>
+      <c r="A104" s="13" t="inlineStr">
+        <is>
+          <t>Queso Crema</t>
         </is>
       </c>
       <c r="B104" s="11" t="n"/>
       <c r="C104" s="11" t="n"/>
-      <c r="D104" s="12" t="n"/>
+      <c r="D104" s="14" t="n"/>
     </row>
     <row r="105" ht="17" customHeight="1">
-      <c r="A105" s="13" t="inlineStr">
-        <is>
-          <t>Queso Panela</t>
+      <c r="A105" s="10" t="inlineStr">
+        <is>
+          <t>Queso Mozzarella</t>
         </is>
       </c>
       <c r="B105" s="11" t="n"/>
       <c r="C105" s="11" t="n"/>
-      <c r="D105" s="14" t="n"/>
+      <c r="D105" s="12" t="n"/>
     </row>
     <row r="106" ht="17" customHeight="1">
-      <c r="A106" s="10" t="inlineStr">
-        <is>
-          <t>Queso Parmesano</t>
+      <c r="A106" s="13" t="inlineStr">
+        <is>
+          <t>Queso Panela</t>
         </is>
       </c>
       <c r="B106" s="11" t="n"/>
       <c r="C106" s="11" t="n"/>
-      <c r="D106" s="12" t="n"/>
+      <c r="D106" s="14" t="n"/>
     </row>
     <row r="107" ht="17" customHeight="1">
-      <c r="A107" s="13" t="inlineStr">
+      <c r="A107" s="10" t="inlineStr">
         <is>
           <t>Queso para Pastas</t>
         </is>
       </c>
       <c r="B107" s="11" t="n"/>
       <c r="C107" s="11" t="n"/>
-      <c r="D107" s="14" t="n"/>
+      <c r="D107" s="12" t="n"/>
     </row>
     <row r="108" ht="17" customHeight="1">
-      <c r="A108" s="10" t="inlineStr">
-        <is>
-          <t>Sal</t>
+      <c r="A108" s="13" t="inlineStr">
+        <is>
+          <t>Queso Parmesano</t>
         </is>
       </c>
       <c r="B108" s="11" t="n"/>
       <c r="C108" s="11" t="n"/>
-      <c r="D108" s="12" t="n"/>
+      <c r="D108" s="14" t="n"/>
     </row>
     <row r="109" ht="17" customHeight="1">
-      <c r="A109" s="13" t="inlineStr">
-        <is>
-          <t>Sal de Mar</t>
+      <c r="A109" s="10" t="inlineStr">
+        <is>
+          <t>Sal</t>
         </is>
       </c>
       <c r="B109" s="11" t="n"/>
       <c r="C109" s="11" t="n"/>
-      <c r="D109" s="14" t="n"/>
+      <c r="D109" s="12" t="n"/>
     </row>
     <row r="110" ht="17" customHeight="1">
-      <c r="A110" s="10" t="inlineStr">
-        <is>
-          <t>Salsa Sriracha</t>
+      <c r="A110" s="13" t="inlineStr">
+        <is>
+          <t>Sal de Mar</t>
         </is>
       </c>
       <c r="B110" s="11" t="n"/>
       <c r="C110" s="11" t="n"/>
-      <c r="D110" s="12" t="n"/>
+      <c r="D110" s="14" t="n"/>
     </row>
     <row r="111" ht="17" customHeight="1">
-      <c r="A111" s="13" t="inlineStr">
-        <is>
-          <t>Tomate pelado</t>
+      <c r="A111" s="10" t="inlineStr">
+        <is>
+          <t>Salsa Sriracha</t>
         </is>
       </c>
       <c r="B111" s="11" t="n"/>
       <c r="C111" s="11" t="n"/>
-      <c r="D111" s="14" t="n"/>
+      <c r="D111" s="12" t="n"/>
     </row>
     <row r="112" ht="17" customHeight="1">
-      <c r="A112" s="10" t="inlineStr">
+      <c r="A112" s="13" t="inlineStr">
         <is>
           <t>Tomate Deshidratado</t>
         </is>
       </c>
       <c r="B112" s="11" t="n"/>
       <c r="C112" s="11" t="n"/>
-      <c r="D112" s="12" t="n"/>
+      <c r="D112" s="14" t="n"/>
     </row>
     <row r="113" ht="17" customHeight="1">
-      <c r="A113" s="13" t="inlineStr">
-        <is>
-          <t>Vainilla</t>
+      <c r="A113" s="10" t="inlineStr">
+        <is>
+          <t>Tomate pelado</t>
         </is>
       </c>
       <c r="B113" s="11" t="n"/>
       <c r="C113" s="11" t="n"/>
-      <c r="D113" s="14" t="n"/>
+      <c r="D113" s="12" t="n"/>
     </row>
     <row r="114" ht="17" customHeight="1">
-      <c r="A114" s="10" t="inlineStr">
-        <is>
-          <t>Vinagre Balsámico</t>
+      <c r="A114" s="13" t="inlineStr">
+        <is>
+          <t>Vainilla</t>
         </is>
       </c>
       <c r="B114" s="11" t="n"/>
       <c r="C114" s="11" t="n"/>
-      <c r="D114" s="12" t="n"/>
+      <c r="D114" s="14" t="n"/>
     </row>
     <row r="115" ht="17" customHeight="1">
-      <c r="A115" s="13" t="inlineStr">
-        <is>
-          <t>Vinagre Blanco</t>
+      <c r="A115" s="10" t="inlineStr">
+        <is>
+          <t>Vinagre Balsámico</t>
         </is>
       </c>
       <c r="B115" s="11" t="n"/>
       <c r="C115" s="11" t="n"/>
-      <c r="D115" s="14" t="n"/>
+      <c r="D115" s="12" t="n"/>
     </row>
     <row r="116" ht="17" customHeight="1">
-      <c r="A116" s="10" t="inlineStr">
-        <is>
-          <t>Vino Blanco</t>
+      <c r="A116" s="13" t="inlineStr">
+        <is>
+          <t>Vinagre Blanco</t>
         </is>
       </c>
       <c r="B116" s="11" t="n"/>
       <c r="C116" s="11" t="n"/>
-      <c r="D116" s="12" t="n"/>
+      <c r="D116" s="14" t="n"/>
     </row>
     <row r="117" ht="17" customHeight="1">
-      <c r="A117" s="13" t="inlineStr">
-        <is>
-          <t>Vino Tinto</t>
+      <c r="A117" s="10" t="inlineStr">
+        <is>
+          <t>Vino Blanco</t>
         </is>
       </c>
       <c r="B117" s="11" t="n"/>
       <c r="C117" s="11" t="n"/>
-      <c r="D117" s="14" t="n"/>
+      <c r="D117" s="12" t="n"/>
     </row>
     <row r="118" ht="17" customHeight="1">
-      <c r="A118" s="10" t="inlineStr">
-        <is>
-          <t>Vitafil</t>
+      <c r="A118" s="13" t="inlineStr">
+        <is>
+          <t>Vino Tinto</t>
         </is>
       </c>
       <c r="B118" s="11" t="n"/>
       <c r="C118" s="11" t="n"/>
-      <c r="D118" s="12" t="n"/>
+      <c r="D118" s="14" t="n"/>
     </row>
     <row r="119" ht="17" customHeight="1">
-      <c r="A119" s="13" t="inlineStr">
-        <is>
-          <t>Yogurt Natural</t>
+      <c r="A119" s="10" t="inlineStr">
+        <is>
+          <t>Vitafil</t>
         </is>
       </c>
       <c r="B119" s="11" t="n"/>
       <c r="C119" s="11" t="n"/>
-      <c r="D119" s="14" t="n"/>
+      <c r="D119" s="12" t="n"/>
     </row>
     <row r="120" ht="17" customHeight="1">
-      <c r="A120" s="10" t="inlineStr"/>
+      <c r="A120" s="13" t="inlineStr">
+        <is>
+          <t>Yogurt Natural</t>
+        </is>
+      </c>
       <c r="B120" s="11" t="n"/>
       <c r="C120" s="11" t="n"/>
-      <c r="D120" s="12" t="n"/>
+      <c r="D120" s="14" t="n"/>
     </row>
     <row r="121" ht="17" customHeight="1">
-      <c r="A121" s="13" t="inlineStr"/>
+      <c r="A121" s="10" t="inlineStr"/>
       <c r="B121" s="11" t="n"/>
       <c r="C121" s="11" t="n"/>
-      <c r="D121" s="14" t="n"/>
-    </row>
-    <row r="122" ht="19" customHeight="1">
-      <c r="A122" s="8" t="inlineStr">
+      <c r="D121" s="12" t="n"/>
+    </row>
+    <row r="122" ht="17" customHeight="1">
+      <c r="A122" s="13" t="inlineStr"/>
+      <c r="B122" s="11" t="n"/>
+      <c r="C122" s="11" t="n"/>
+      <c r="D122" s="14" t="n"/>
+    </row>
+    <row r="123" ht="19" customHeight="1">
+      <c r="A123" s="8" t="inlineStr">
         <is>
           <t>LIMPIEZA</t>
         </is>
       </c>
-      <c r="B122" s="9" t="n"/>
-      <c r="C122" s="9" t="n"/>
-      <c r="D122" s="9" t="n"/>
-    </row>
-    <row r="123" ht="17" customHeight="1">
-      <c r="A123" s="10" t="inlineStr">
+      <c r="B123" s="9" t="n"/>
+      <c r="C123" s="9" t="n"/>
+      <c r="D123" s="9" t="n"/>
+    </row>
+    <row r="124" ht="17" customHeight="1">
+      <c r="A124" s="10" t="inlineStr">
         <is>
           <t>Bolsa camiseta</t>
-        </is>
-      </c>
-      <c r="B123" s="11" t="n"/>
-      <c r="C123" s="11" t="n"/>
-      <c r="D123" s="12" t="n"/>
-    </row>
-    <row r="124" ht="17" customHeight="1">
-      <c r="A124" s="13" t="inlineStr">
-        <is>
-          <t>Bolsas 1/2 k</t>
         </is>
       </c>
       <c r="B124" s="11" t="n"/>
       <c r="C124" s="11" t="n"/>
-      <c r="D124" s="14" t="n"/>
+      <c r="D124" s="12" t="n"/>
     </row>
     <row r="125" ht="17" customHeight="1">
-      <c r="A125" s="10" t="inlineStr">
+      <c r="A125" s="13" t="inlineStr">
         <is>
           <t>Bolsas 1 k</t>
         </is>
       </c>
       <c r="B125" s="11" t="n"/>
       <c r="C125" s="11" t="n"/>
-      <c r="D125" s="12" t="n"/>
+      <c r="D125" s="14" t="n"/>
     </row>
     <row r="126" ht="17" customHeight="1">
-      <c r="A126" s="13" t="inlineStr">
-        <is>
-          <t>Bolsas 3 k</t>
+      <c r="A126" s="10" t="inlineStr">
+        <is>
+          <t>Bolsas 1/2 k</t>
         </is>
       </c>
       <c r="B126" s="11" t="n"/>
       <c r="C126" s="11" t="n"/>
-      <c r="D126" s="14" t="n"/>
+      <c r="D126" s="12" t="n"/>
     </row>
     <row r="127" ht="17" customHeight="1">
-      <c r="A127" s="10" t="inlineStr">
-        <is>
-          <t>Bolsas de basura N.</t>
+      <c r="A127" s="13" t="inlineStr">
+        <is>
+          <t>Bolsas 3 k</t>
         </is>
       </c>
       <c r="B127" s="11" t="n"/>
       <c r="C127" s="11" t="n"/>
-      <c r="D127" s="12" t="n"/>
+      <c r="D127" s="14" t="n"/>
     </row>
     <row r="128" ht="17" customHeight="1">
-      <c r="A128" s="13" t="inlineStr">
-        <is>
-          <t>Caja pizza 16</t>
+      <c r="A128" s="10" t="inlineStr">
+        <is>
+          <t>Bolsas de basura N.</t>
         </is>
       </c>
       <c r="B128" s="11" t="n"/>
       <c r="C128" s="11" t="n"/>
-      <c r="D128" s="14" t="n"/>
+      <c r="D128" s="12" t="n"/>
     </row>
     <row r="129" ht="17" customHeight="1">
-      <c r="A129" s="10" t="inlineStr">
+      <c r="A129" s="13" t="inlineStr">
         <is>
           <t>Caja pizza 12</t>
         </is>
       </c>
       <c r="B129" s="11" t="n"/>
       <c r="C129" s="11" t="n"/>
-      <c r="D129" s="12" t="n"/>
+      <c r="D129" s="14" t="n"/>
     </row>
     <row r="130" ht="17" customHeight="1">
-      <c r="A130" s="13" t="inlineStr">
-        <is>
-          <t>Cloro</t>
+      <c r="A130" s="10" t="inlineStr">
+        <is>
+          <t>Caja pizza 16</t>
         </is>
       </c>
       <c r="B130" s="11" t="n"/>
       <c r="C130" s="11" t="n"/>
-      <c r="D130" s="14" t="n"/>
+      <c r="D130" s="12" t="n"/>
     </row>
     <row r="131" ht="17" customHeight="1">
-      <c r="A131" s="10" t="inlineStr">
-        <is>
-          <t>Desengrasante</t>
+      <c r="A131" s="13" t="inlineStr">
+        <is>
+          <t>Cloro</t>
         </is>
       </c>
       <c r="B131" s="11" t="n"/>
       <c r="C131" s="11" t="n"/>
-      <c r="D131" s="12" t="n"/>
+      <c r="D131" s="14" t="n"/>
     </row>
     <row r="132" ht="17" customHeight="1">
-      <c r="A132" s="13" t="inlineStr">
-        <is>
-          <t>Escoba</t>
+      <c r="A132" s="10" t="inlineStr">
+        <is>
+          <t>Desengrasante</t>
         </is>
       </c>
       <c r="B132" s="11" t="n"/>
       <c r="C132" s="11" t="n"/>
-      <c r="D132" s="14" t="n"/>
+      <c r="D132" s="12" t="n"/>
     </row>
     <row r="133" ht="17" customHeight="1">
-      <c r="A133" s="10" t="inlineStr">
-        <is>
-          <t>Fabuloso</t>
+      <c r="A133" s="13" t="inlineStr">
+        <is>
+          <t>Escoba</t>
         </is>
       </c>
       <c r="B133" s="11" t="n"/>
       <c r="C133" s="11" t="n"/>
-      <c r="D133" s="12" t="n"/>
+      <c r="D133" s="14" t="n"/>
     </row>
     <row r="134" ht="17" customHeight="1">
-      <c r="A134" s="13" t="inlineStr">
-        <is>
-          <t>Fibras Esponja</t>
+      <c r="A134" s="10" t="inlineStr">
+        <is>
+          <t>Fabuloso</t>
         </is>
       </c>
       <c r="B134" s="11" t="n"/>
       <c r="C134" s="11" t="n"/>
-      <c r="D134" s="14" t="n"/>
+      <c r="D134" s="12" t="n"/>
     </row>
     <row r="135" ht="17" customHeight="1">
-      <c r="A135" s="10" t="inlineStr">
-        <is>
-          <t>Fibras Metal</t>
+      <c r="A135" s="13" t="inlineStr">
+        <is>
+          <t>Fibras Esponja</t>
         </is>
       </c>
       <c r="B135" s="11" t="n"/>
       <c r="C135" s="11" t="n"/>
-      <c r="D135" s="12" t="n"/>
+      <c r="D135" s="14" t="n"/>
     </row>
     <row r="136" ht="17" customHeight="1">
-      <c r="A136" s="13" t="inlineStr">
-        <is>
-          <t>Franela</t>
+      <c r="A136" s="10" t="inlineStr">
+        <is>
+          <t>Fibras Metal</t>
         </is>
       </c>
       <c r="B136" s="11" t="n"/>
       <c r="C136" s="11" t="n"/>
-      <c r="D136" s="14" t="n"/>
+      <c r="D136" s="12" t="n"/>
     </row>
     <row r="137" ht="17" customHeight="1">
-      <c r="A137" s="10" t="inlineStr">
-        <is>
-          <t>Jabón para Trastes</t>
+      <c r="A137" s="13" t="inlineStr">
+        <is>
+          <t>Franela</t>
         </is>
       </c>
       <c r="B137" s="11" t="n"/>
       <c r="C137" s="11" t="n"/>
-      <c r="D137" s="12" t="n"/>
+      <c r="D137" s="14" t="n"/>
     </row>
     <row r="138" ht="17" customHeight="1">
-      <c r="A138" s="13" t="inlineStr">
-        <is>
-          <t>Recogedor</t>
+      <c r="A138" s="10" t="inlineStr">
+        <is>
+          <t>Jabón para Trastes</t>
         </is>
       </c>
       <c r="B138" s="11" t="n"/>
       <c r="C138" s="11" t="n"/>
-      <c r="D138" s="14" t="n"/>
+      <c r="D138" s="12" t="n"/>
     </row>
     <row r="139" ht="17" customHeight="1">
-      <c r="A139" s="10" t="inlineStr">
-        <is>
-          <t>Trapeador</t>
+      <c r="A139" s="13" t="inlineStr">
+        <is>
+          <t>Recogedor</t>
         </is>
       </c>
       <c r="B139" s="11" t="n"/>
       <c r="C139" s="11" t="n"/>
-      <c r="D139" s="12" t="n"/>
+      <c r="D139" s="14" t="n"/>
     </row>
     <row r="140" ht="17" customHeight="1">
-      <c r="A140" s="13" t="inlineStr"/>
+      <c r="A140" s="10" t="inlineStr">
+        <is>
+          <t>Trapeador</t>
+        </is>
+      </c>
       <c r="B140" s="11" t="n"/>
       <c r="C140" s="11" t="n"/>
-      <c r="D140" s="14" t="n"/>
+      <c r="D140" s="12" t="n"/>
     </row>
     <row r="141" ht="17" customHeight="1">
-      <c r="A141" s="10" t="inlineStr"/>
+      <c r="A141" s="13" t="inlineStr"/>
       <c r="B141" s="11" t="n"/>
       <c r="C141" s="11" t="n"/>
-      <c r="D141" s="12" t="n"/>
+      <c r="D141" s="14" t="n"/>
+    </row>
+    <row r="142" ht="17" customHeight="1">
+      <c r="A142" s="10" t="inlineStr"/>
+      <c r="B142" s="11" t="n"/>
+      <c r="C142" s="11" t="n"/>
+      <c r="D142" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A56:D56"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="A8:D8"/>
     <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A122:D122"/>
     <mergeCell ref="A35:D35"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="B4:D4"/>
-    <mergeCell ref="A55:D55"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A123:D123"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>